<commit_message>
msm: split demo screenshots into pages, update docs and demo scripts
</commit_message>
<xml_diff>
--- a/msm/demo/msm_protocol.xlsx
+++ b/msm/demo/msm_protocol.xlsx
@@ -42,25 +42,25 @@
     <t>description</t>
   </si>
   <si>
-    <t>Adults aged 18+</t>
+    <t>Adults followed for 10 discrete periods (N=500; 5000 person-period observations)</t>
   </si>
   <si>
-    <t>Binary drug exposure (treated vs untreated)</t>
+    <t>Dynamic treatment assignment at each period; counterfactual contrast is always treated versus never treated</t>
   </si>
   <si>
-    <t>Biomarker, comorbidity, age, sex</t>
+    <t>Time-varying: biomarker, comorbidity; baseline: age, sex; informative censoring indicator</t>
   </si>
   <si>
-    <t>Binary outcome (event/no event)</t>
+    <t>Binary outcome assessed each period and summarized as cumulative incidence over follow-up</t>
   </si>
   <si>
-    <t>ATE: E[Y(1)] - E[Y(0)]</t>
+    <t>Risk difference in cumulative incidence under always-treated versus never-treated strategies</t>
   </si>
   <si>
-    <t>Stabilized IPTW, numerator: age sex, denominator: biomarker comorbidity age sex</t>
+    <t>Stabilized IPTW with baseline numerator model, denominator model including time-varying covariates, and 1st/99th percentile truncation</t>
   </si>
   <si>
-    <t>Weighted pooled logistic regression with quadratic period</t>
+    <t>Validated pooled logistic MSM with quadratic time trend, robust SEs, Monte Carlo prediction intervals, and E-value sensitivity analysis</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
finegray: add goodness-of-fit and nuisance-model QA suite
</commit_message>
<xml_diff>
--- a/msm/demo/msm_protocol.xlsx
+++ b/msm/demo/msm_protocol.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="32" uniqueCount="17">
   <si>
     <t>component</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>Validated pooled logistic MSM with quadratic time trend, robust SEs, Monte Carlo prediction intervals, and E-value sensitivity analysis</t>
+  </si>
+  <si>
+    <t>Adults followed for 10 discrete periods (N=500; 4586 person-period observations)</t>
   </si>
 </sst>
 </file>
@@ -120,7 +123,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">

</xml_diff>